<commit_message>
pay roll push 2
</commit_message>
<xml_diff>
--- a/files/Sample_Payroll.xlsx
+++ b/files/Sample_Payroll.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Payroll" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,29 +397,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH3"/>
+  <dimension ref="A1:AM3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>S.No.</v>
       </c>
       <c r="B1" t="str">
+        <v>Emp Id</v>
+      </c>
+      <c r="C1" t="str">
         <v>Name of the staff</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Dept</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Designation</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Date of joining</v>
       </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
       <c r="G1" t="str">
-        <v/>
+        <v>Allowances</v>
       </c>
       <c r="H1" t="str">
         <v/>
@@ -452,17 +452,17 @@
         <v/>
       </c>
       <c r="R1" t="str">
+        <v>Addl maint. Salary</v>
+      </c>
+      <c r="S1" t="str">
         <v>No. of LOP</v>
       </c>
-      <c r="S1" t="str">
-        <v/>
-      </c>
       <c r="T1" t="str">
+        <v>No. of OD in days</v>
+      </c>
+      <c r="U1" t="str">
         <v>Deduction</v>
       </c>
-      <c r="U1" t="str">
-        <v/>
-      </c>
       <c r="V1" t="str">
         <v/>
       </c>
@@ -485,21 +485,36 @@
         <v/>
       </c>
       <c r="AC1" t="str">
+        <v/>
+      </c>
+      <c r="AD1" t="str">
+        <v/>
+      </c>
+      <c r="AE1" t="str">
+        <v>Salary after deduction</v>
+      </c>
+      <c r="AF1" t="str">
         <v>Total Deduction</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AG1" t="str">
         <v>Advance</v>
       </c>
-      <c r="AE1" t="str">
-        <v/>
-      </c>
-      <c r="AF1" t="str">
-        <v/>
-      </c>
-      <c r="AG1" t="str">
+      <c r="AH1" t="str">
+        <v/>
+      </c>
+      <c r="AI1" t="str">
+        <v/>
+      </c>
+      <c r="AJ1" t="str">
+        <v>Addition</v>
+      </c>
+      <c r="AK1" t="str">
+        <v/>
+      </c>
+      <c r="AL1" t="str">
         <v>Net Salary</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AM1" t="str">
         <v/>
       </c>
     </row>
@@ -562,69 +577,84 @@
         <v/>
       </c>
       <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
         <v>LOP</v>
       </c>
-      <c r="U2" t="str">
+      <c r="V2" t="str">
         <v>Hostel</v>
       </c>
-      <c r="V2" t="str">
+      <c r="W2" t="str">
         <v>Trans.</v>
       </c>
-      <c r="W2" t="str">
+      <c r="X2" t="str">
         <v>EPF(1)</v>
       </c>
-      <c r="X2" t="str">
+      <c r="Y2" t="str">
         <v>EPF(2)</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="Z2" t="str">
         <v>ESI</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AA2" t="str">
         <v>TDS</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AB2" t="str">
         <v>Prof.Tax</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AC2" t="str">
         <v>Medical</v>
       </c>
-      <c r="AC2" t="str">
-        <v/>
-      </c>
       <c r="AD2" t="str">
+        <v>Others</v>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
         <v>Paid</v>
       </c>
-      <c r="AE2" t="str">
+      <c r="AH2" t="str">
         <v>Recd</v>
       </c>
-      <c r="AF2" t="str">
+      <c r="AI2" t="str">
         <v>Bal</v>
       </c>
-      <c r="AG2" t="str">
-        <v/>
-      </c>
-      <c r="AH2" t="str">
-        <v/>
+      <c r="AJ2" t="str">
+        <v>OD amt</v>
+      </c>
+      <c r="AK2" t="str">
+        <v>Maiint.amt</v>
+      </c>
+      <c r="AL2" t="str">
+        <v>By Bank</v>
+      </c>
+      <c r="AM2" t="str">
+        <v>By cash</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="str">
         <v>SECETCS002</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Test Employee</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Computer Science</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Assistant Professor</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>2022-06-01</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
       </c>
       <c r="G3">
         <v>50000</v>
@@ -662,8 +692,8 @@
       <c r="R3">
         <v>0</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
+      <c r="S3">
+        <v>0</v>
       </c>
       <c r="T3">
         <v>0</v>
@@ -675,45 +705,60 @@
         <v>0</v>
       </c>
       <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
         <v>1800</v>
       </c>
-      <c r="X3">
-        <v>0</v>
-      </c>
       <c r="Y3">
         <v>0</v>
       </c>
       <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
         <v>500</v>
       </c>
-      <c r="AA3">
+      <c r="AB3">
         <v>200</v>
       </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
       <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>64300</v>
+      </c>
+      <c r="AF3">
         <v>2500</v>
       </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3">
-        <v>0</v>
-      </c>
-      <c r="AF3">
-        <v>0</v>
-      </c>
       <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>0</v>
+      </c>
+      <c r="AJ3">
+        <v>0</v>
+      </c>
+      <c r="AK3">
+        <v>0</v>
+      </c>
+      <c r="AL3">
         <v>64300</v>
       </c>
-      <c r="AH3" t="str">
-        <v/>
+      <c r="AM3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>